<commit_message>
Regenerate verified case artifacts with native binning figures
</commit_message>
<xml_diff>
--- a/docs/assets/cases/policy.xlsx
+++ b/docs/assets/cases/policy.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="FeatureMetadata" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="BusinessContext" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ReportSemantics" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="000_summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="001_regions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="002_changes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="003_cell_decisions" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="004_bins" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FeatureMetadata" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BusinessContext" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReportSemantics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000_summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="001_regions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="002_changes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="003_cell_decisions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="004_bins" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -732,7 +732,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>"df121489-258c-4b99-9338-c88759598869"</t>
+          <t>"4154620a-048d-4437-b18c-c4dacc008dd9"</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"score_x":"main_score","score_y":"aux_score","score_directions":{"main_score":"lower_risk","aux_score":"higher_risk"},"targets":["bad30","late60"],"requested_n_bins":5,"actual_n_bins":{"main_score":4,"aux_score":4},"bin_definitions":{"x":{"score":"main_score","direction":"lower_risk","cutpoints":[546.042988729658,601.2262132556998,653.7750315986514],"special_values":[],"probability":false,"closed":"right","actual_n_bins":4,"fit":{"binning_type":"native","binner_params":{"cart_params":{},"join_threshold":100,"merge_small_bins":false,"method":"quantile","min_bin_size":0.05,"missing_values":[],"n_bins":4,"n_jobs":-1,"remove_empty_bins":false,"special_values":[]},"source":"current_input","target":null,"reference_row_count":6000,"valid_score_row_count":5971,"fit_row_count":6000,"usable_fit_row_count":5971,"observed_class_count":null,"requested_n_bins":4,"actual_n_bins":4,"diagnostic":null,"fitted_trend":null,"closed":"right"}},"y":{"score":"aux_score","direction":"higher_risk","cutpoints":[432.41255966198844,498.7917609295865,567.1738809810513],"special_values":[-999],"probability":false,"closed":"right","actual_n_bins":4,"fit":{"binning_type":"native","binner_params":{"cart_params":{},"join_threshold":100,"merge_small_bins":false,"method":"quantile","min_bin_size":0.05,"missing_values":[],"n_bins":4,"n_jobs":-1,"remove_empty_bins":false,"special_values":[-999]},"source":"current_input","target":null,"reference_row_count":6000,"valid_score_row_count":5910,"fit_row_count":6000,"usable_fit_row_count":5910,"observed_class_count":null,"requested_n_bins":4,"actual_n_bins":4,"diagnostic":null,"fitted_trend":null,"closed":"right"}}},"binning_type":null,"binning_target":null,"fitted_targets":{"x":null,"y":null},"fit_performed":false,"binning_parameters":{"x":{"binning_type":"native","binner_params":{"cart_params":{},"join_threshold":100,"merge_small_bins":false,"method":"quantile","min_bin_size":0.05,"missing_values":[],"n_bins":4,"n_jobs":-1,"remove_empty_bins":false,"special_values":[]},"source":"current_input","target":null,"reference_row_count":6000,"valid_score_row_count":5971,"fit_row_count":6000,"usable_fit_row_count":5971,"observed_class_count":null,"requested_n_bins":4,"actual_n_bins":4,"diagnostic":null,"fitted_trend":null,"closed":"right"},"y":{"binning_type":"native","binner_params":{"cart_params":{},"join_threshold":100,"merge_small_bins":false,"method":"quantile","min_bin_size":0.05,"missing_values":[],"n_bins":4,"n_jobs":-1,"remove_empty_bins":false,"special_values":[-999]},"source":"current_input","target":null,"reference_row_count":6000,"valid_score_row_count":5910,"fit_row_count":6000,"usable_fit_row_count":5910,"observed_class_count":null,"requested_n_bins":4,"actual_n_bins":4,"diagnostic":null,"fitted_trend":null,"closed":"right"}},"binning_reference_policy":"explicit reference or current input; fitted once per axis across all scopes/targets","fit_source":"saved_definition","input_row_count":18000,"projected_columns":["main_score","aux_score","bad30","late60","dataset","application_date","weight","amount"],"group_col":"dataset","time_col":"application_date","time_grain":"month","scope_dimensions":{"group":{"source":"group","column":"dataset","grain":null},"period":{"source":"time","column":"application_date","grain":"month"}},"actual_scope_count":9,"max_scopes":10000,"weights_col":"weight","amount_col":"amount","min_observed":30,"confidence_level":0.95,"sample_share_denominator":"all samples including special bins, per target/group/period","bad_rate_denominator":"observed_weight_sum","confidence_interval":"unweighted integer Wilson; weighted CI unsupported","amount_policy":"existing helper: nonnegative amounts contribute; negative/null/NaN contribute zero; infinity rejected","score_missing_policy":"null/NaN/custom missing_values -&gt; missing; nonfinite/nonnumeric/probability domain violation -&gt; invalid","ratio_unit":"fraction; delta fraction difference","sample_semantics":"historical sample retention; population extrapolation unknown","parent_report_id":"066dccc0-b803-4f2a-8f3c-2ace86cf0ada","candidate":{"missing_score":"reject","type":"expression","expression":"X &lt;= X2 AND Y &lt;= Y2"},"baseline":{"missing_score":"reject","type":"x_only","x_max_risk_rank":2},"replay_precision":"exact whole saved bins only","comparison":"historical sample retention; coverage differences explicit","candidate_expression_ast":{"kind":"and","operands":[{"kind":"compare","axis":"X","operator":"&lt;=","rank":2},{"kind":"compare","axis":"Y","operator":"&lt;=","rank":2}]},"expression_syntax":{"version":1,"limits":{"max_length":240,"max_tokens":96,"max_depth":12},"normal_bins_only":true,"ordering":"saved risk_rank ascending, stable across target/group/period"}}</t>
+          <t>{"score_x":"main_score","score_y":"aux_score","score_directions":{"main_score":"lower_risk","aux_score":"higher_risk"},"targets":["bad30","late60"],"requested_n_bins":5,"actual_n_bins":{"main_score":4,"aux_score":4},"bin_definitions":{"x":{"score":"main_score","direction":"lower_risk","cutpoints":[546.042988729658,601.2262132556998,653.7750315986514],"special_values":[],"probability":false,"closed":"right","actual_n_bins":4,"fit":{"binning_type":"native","binner_params":{"cart_params":{},"join_threshold":100,"merge_small_bins":false,"method":"quantile","min_bin_size":0.05,"missing_values":[],"n_bins":4,"n_jobs":-1,"remove_empty_bins":false,"special_values":[]},"source":"current_input","target":null,"reference_row_count":6000,"valid_score_row_count":5971,"fit_row_count":6000,"usable_fit_row_count":5971,"observed_class_count":null,"requested_n_bins":4,"actual_n_bins":4,"diagnostic":null,"fitted_trend":null,"closed":"right"}},"y":{"score":"aux_score","direction":"higher_risk","cutpoints":[432.41255966198844,498.7917609295865,567.1738809810513],"special_values":[-999],"probability":false,"closed":"right","actual_n_bins":4,"fit":{"binning_type":"native","binner_params":{"cart_params":{},"join_threshold":100,"merge_small_bins":false,"method":"quantile","min_bin_size":0.05,"missing_values":[],"n_bins":4,"n_jobs":-1,"remove_empty_bins":false,"special_values":[-999]},"source":"current_input","target":null,"reference_row_count":6000,"valid_score_row_count":5910,"fit_row_count":6000,"usable_fit_row_count":5910,"observed_class_count":null,"requested_n_bins":4,"actual_n_bins":4,"diagnostic":null,"fitted_trend":null,"closed":"right"}}},"binning_type":null,"binning_target":null,"fitted_targets":{"x":null,"y":null},"fit_performed":false,"binning_parameters":{"x":{"binning_type":"native","binner_params":{"cart_params":{},"join_threshold":100,"merge_small_bins":false,"method":"quantile","min_bin_size":0.05,"missing_values":[],"n_bins":4,"n_jobs":-1,"remove_empty_bins":false,"special_values":[]},"source":"current_input","target":null,"reference_row_count":6000,"valid_score_row_count":5971,"fit_row_count":6000,"usable_fit_row_count":5971,"observed_class_count":null,"requested_n_bins":4,"actual_n_bins":4,"diagnostic":null,"fitted_trend":null,"closed":"right"},"y":{"binning_type":"native","binner_params":{"cart_params":{},"join_threshold":100,"merge_small_bins":false,"method":"quantile","min_bin_size":0.05,"missing_values":[],"n_bins":4,"n_jobs":-1,"remove_empty_bins":false,"special_values":[-999]},"source":"current_input","target":null,"reference_row_count":6000,"valid_score_row_count":5910,"fit_row_count":6000,"usable_fit_row_count":5910,"observed_class_count":null,"requested_n_bins":4,"actual_n_bins":4,"diagnostic":null,"fitted_trend":null,"closed":"right"}},"binning_reference_policy":"explicit reference or current input; fitted once per axis across all scopes/targets","fit_source":"saved_definition","input_row_count":18000,"projected_columns":["main_score","aux_score","bad30","late60","dataset","application_date","weight","amount"],"group_col":"dataset","time_col":"application_date","time_grain":"month","scope_dimensions":{"group":{"source":"group","column":"dataset","grain":null},"period":{"source":"time","column":"application_date","grain":"month"}},"actual_scope_count":9,"max_scopes":10000,"weights_col":"weight","amount_col":"amount","min_observed":30,"confidence_level":0.95,"sample_share_denominator":"all samples including special bins, per target/group/period","bad_rate_denominator":"observed_weight_sum","confidence_interval":"unweighted integer Wilson; weighted CI unsupported","amount_policy":"existing helper: nonnegative amounts contribute; negative/null/NaN contribute zero; infinity rejected","score_missing_policy":"null/NaN/custom missing_values -&gt; missing; nonfinite/nonnumeric/probability domain violation -&gt; invalid","ratio_unit":"fraction; delta fraction difference","sample_semantics":"historical sample retention; population extrapolation unknown","parent_report_id":"cba02fb3-e2e3-44ae-8c72-32ab920fd80c","candidate":{"missing_score":"reject","type":"expression","expression":"X &lt;= X2 AND Y &lt;= Y2"},"baseline":{"missing_score":"reject","type":"x_only","x_max_risk_rank":2},"replay_precision":"exact whole saved bins only","comparison":"historical sample retention; coverage differences explicit","candidate_expression_ast":{"kind":"and","operands":[{"kind":"compare","axis":"X","operator":"&lt;=","rank":2},{"kind":"compare","axis":"Y","operator":"&lt;=","rank":2}]},"expression_syntax":{"version":1,"limits":{"max_length":240,"max_tokens":96,"max_depth":12},"normal_bins_only":true,"ordering":"saved risk_rank ascending, stable across target/group/period"}}</t>
         </is>
       </c>
     </row>

</xml_diff>